<commit_message>
fix(prod): weather GPS resolution, admin broadcast history & recipient tracking, read receipts, and system health
</commit_message>
<xml_diff>
--- a/backend/tests/api_test_results.xlsx
+++ b/backend/tests/api_test_results.xlsx
@@ -429,7 +429,7 @@
         <v>Execution Time</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-27T15:56:11.294Z</v>
+        <v>2026-10-31T04:17:20.374Z</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>Duration (s)</v>
       </c>
       <c r="B9" t="str">
-        <v>35.28</v>
+        <v>58.98</v>
       </c>
     </row>
   </sheetData>
@@ -514,7 +514,7 @@
         <v>PASS</v>
       </c>
       <c r="D2">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E2" t="str">
         <v>Liveness probe healthy (HTTP 200)</v>
@@ -531,7 +531,7 @@
         <v>PASS</v>
       </c>
       <c r="D3">
-        <v>934</v>
+        <v>5278</v>
       </c>
       <c r="E3" t="str">
         <v>Database connection pool active &amp; healthy</v>
@@ -548,7 +548,7 @@
         <v>PASS</v>
       </c>
       <c r="D4">
-        <v>1736</v>
+        <v>3610</v>
       </c>
       <c r="E4" t="str">
         <v>Correctly rejected invalid login with HTTP 401</v>
@@ -565,7 +565,7 @@
         <v>PASS</v>
       </c>
       <c r="D5">
-        <v>1103</v>
+        <v>1637</v>
       </c>
       <c r="E5" t="str">
         <v>Authenticated successfully as farmer.live@agrorent.ai (JWT token issued)</v>
@@ -582,7 +582,7 @@
         <v>PASS</v>
       </c>
       <c r="D6">
-        <v>2248</v>
+        <v>1825</v>
       </c>
       <c r="E6" t="str">
         <v>Authenticated successfully as owner.demo@agrorent.ai (JWT token issued)</v>
@@ -599,7 +599,7 @@
         <v>PASS</v>
       </c>
       <c r="D7">
-        <v>2050</v>
+        <v>4590</v>
       </c>
       <c r="E7" t="str">
         <v>Returned 20 equipment machinery items</v>
@@ -616,10 +616,10 @@
         <v>PASS</v>
       </c>
       <c r="D8">
-        <v>1149</v>
+        <v>2294</v>
       </c>
       <c r="E8" t="str">
-        <v>Geographic proximity search active (0 items found)</v>
+        <v>Geographic proximity search active (1 items found)</v>
       </c>
     </row>
     <row r="9">
@@ -633,7 +633,7 @@
         <v>PASS</v>
       </c>
       <c r="D9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="str">
         <v>Category taxonomy verified (8 categories available)</v>
@@ -650,7 +650,7 @@
         <v>PASS</v>
       </c>
       <c r="D10">
-        <v>5127</v>
+        <v>7736</v>
       </c>
       <c r="E10" t="str">
         <v>Retrieved user rental booking list successfully (4 bookings)</v>
@@ -667,7 +667,7 @@
         <v>PASS</v>
       </c>
       <c r="D11">
-        <v>2611</v>
+        <v>4222</v>
       </c>
       <c r="E11" t="str">
         <v>Retrieved digital twin farm records (1 farms registered)</v>
@@ -684,7 +684,7 @@
         <v>PASS</v>
       </c>
       <c r="D12">
-        <v>1852</v>
+        <v>2442</v>
       </c>
       <c r="E12" t="str">
         <v>Retrieved saved IDs list (0 bookmarks)</v>
@@ -701,7 +701,7 @@
         <v>PASS</v>
       </c>
       <c r="D13">
-        <v>3935</v>
+        <v>6321</v>
       </c>
       <c r="E13" t="str">
         <v>Owner dashboard KPIs, revenue metrics, and booking counts returned</v>
@@ -718,7 +718,7 @@
         <v>PASS</v>
       </c>
       <c r="D14">
-        <v>1741</v>
+        <v>3303</v>
       </c>
       <c r="E14" t="str">
         <v>Retrieved bank details with masked security: Configured</v>
@@ -735,7 +735,7 @@
         <v>PASS</v>
       </c>
       <c r="D15">
-        <v>2527</v>
+        <v>4175</v>
       </c>
       <c r="E15" t="str">
         <v>Community metadata verified: AgroRent Farmer Community</v>
@@ -752,7 +752,7 @@
         <v>PASS</v>
       </c>
       <c r="D16">
-        <v>2062</v>
+        <v>3164</v>
       </c>
       <c r="E16" t="str">
         <v>Retrieved community messages (0 messages loaded)</v>
@@ -769,7 +769,7 @@
         <v>PASS</v>
       </c>
       <c r="D17">
-        <v>6181</v>
+        <v>8361</v>
       </c>
       <c r="E17" t="str">
         <v>AI agronomic advice generated (Fallback active)</v>

</xml_diff>